<commit_message>
07.31날 모든 공정 Sequence Task , Connector 추가 및 수정, 로봇들 좌표 수정
</commit_message>
<xml_diff>
--- a/PLC/IO List.xlsx
+++ b/PLC/IO List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezen-01\Desktop\Project\PLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19097A28-10A3-4342-936B-5164D9DC6526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{704900FD-B174-41EE-8FCC-ADE6621AE164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4920" yWindow="3825" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{E8A3CD3B-D612-4B37-A180-F6C335096DC9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{E8A3CD3B-D612-4B37-A180-F6C335096DC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1206" uniqueCount="890">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="899">
   <si>
     <t>X10</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2584,601 +2584,641 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>2공정(접착제)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6공정(접착제)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8공정(접착제)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>AGV
-P[3]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+P[2~5]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>볼트공급
+P[2]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M300</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M301</t>
+  </si>
+  <si>
+    <t>M302</t>
+  </si>
+  <si>
+    <t>M303</t>
+  </si>
+  <si>
+    <t>M304</t>
+  </si>
+  <si>
+    <t>M305</t>
+  </si>
+  <si>
+    <t>M306</t>
+  </si>
+  <si>
+    <t>M307</t>
+  </si>
+  <si>
+    <t>M308</t>
+  </si>
+  <si>
+    <t>M309</t>
+  </si>
+  <si>
+    <t>M310</t>
+  </si>
+  <si>
+    <t>M311</t>
+  </si>
+  <si>
+    <t>M312</t>
+  </si>
+  <si>
+    <t>M313</t>
+  </si>
+  <si>
+    <t>경화1 공정 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정1 AGV 배출 신호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정1 완료 후 문닫힘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화2 공정 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정2 AGV 배출 신호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정2 완료 후 문닫힘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화3 공정 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정3 AGV 배출 신호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경화공정3 완료 후 문닫힘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M120</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M121</t>
+  </si>
+  <si>
+    <t>M122</t>
+  </si>
+  <si>
+    <t>M123</t>
+  </si>
+  <si>
+    <t>M124</t>
+  </si>
+  <si>
+    <t>M125</t>
+  </si>
+  <si>
+    <t>M126</t>
+  </si>
+  <si>
+    <t>M127</t>
+  </si>
+  <si>
+    <t>M128</t>
+  </si>
+  <si>
+    <t>AGV 내부 펄스</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T21</t>
+  </si>
+  <si>
+    <t>T22</t>
+  </si>
+  <si>
+    <t>T23</t>
+  </si>
+  <si>
+    <t>T24</t>
+  </si>
+  <si>
+    <t>T25</t>
+  </si>
+  <si>
+    <t>T26</t>
+  </si>
+  <si>
+    <t>T27</t>
+  </si>
+  <si>
+    <t>T28</t>
+  </si>
+  <si>
+    <t>T29</t>
+  </si>
+  <si>
+    <t>1공정 agv 신호 딜레이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>3공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>4공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>5공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>6공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>7공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>8공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>9공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>10공정 agv 신호 딜레이</t>
+  </si>
+  <si>
+    <t>M129</t>
+  </si>
+  <si>
+    <t>프레스1(제4공정_저항 검사 공정)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>프레스2(제1공정_하우징 공정)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>로봇1 작업완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>로봇2 작업완료</t>
+  </si>
+  <si>
+    <t>로봇3 작업완료</t>
+  </si>
+  <si>
+    <t>로봇5 작업완료</t>
+  </si>
+  <si>
+    <t>로봇6 작업완료</t>
+  </si>
+  <si>
+    <t>로봇7 작업완료</t>
+  </si>
+  <si>
+    <t>로봇8 작업완료</t>
+  </si>
+  <si>
+    <t>로봇9 작업완료</t>
+  </si>
+  <si>
+    <t>프레스 작업완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>챔버1 상태</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M11</t>
+  </si>
+  <si>
+    <t>M12</t>
+  </si>
+  <si>
+    <t>M13</t>
+  </si>
+  <si>
+    <t>챔버2 상태</t>
+  </si>
+  <si>
+    <t>챔버3 상태</t>
+  </si>
+  <si>
+    <t>챔버4 상태</t>
+  </si>
+  <si>
+    <t>T30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>챔버1 완료 후 딜레이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T31</t>
+  </si>
+  <si>
+    <t>T32</t>
+  </si>
+  <si>
+    <t>T33</t>
+  </si>
+  <si>
+    <t>챔버2 완료 후 딜레이</t>
+  </si>
+  <si>
+    <t>챔버3 완료 후 딜레이</t>
+  </si>
+  <si>
+    <t>챔버4 완료 후 딜레이</t>
+  </si>
+  <si>
+    <t>M15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M16</t>
+  </si>
+  <si>
+    <t>M17</t>
+  </si>
+  <si>
+    <t>M18</t>
+  </si>
+  <si>
+    <t>챔버1 로봇 경유위치 이동 완료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>챔버2 로봇 경유위치 이동 완료</t>
+  </si>
+  <si>
+    <t>챔버3 로봇 경유위치 이동 완료</t>
+  </si>
+  <si>
+    <t>챔버4 로봇 경유위치 이동 완료</t>
+  </si>
+  <si>
+    <t>M20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>수작업7 START</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M21</t>
+  </si>
+  <si>
+    <t>M22</t>
+  </si>
+  <si>
+    <t>수작업8 START</t>
+  </si>
+  <si>
+    <t>수작업9 START</t>
+  </si>
+  <si>
+    <t>출하장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PASS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NG</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M90</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M91</t>
+  </si>
+  <si>
+    <t>M92</t>
+  </si>
+  <si>
+    <t>M93</t>
+  </si>
+  <si>
+    <t>M94</t>
+  </si>
+  <si>
+    <t>M95</t>
+  </si>
+  <si>
+    <t>AGV2</t>
+  </si>
+  <si>
+    <t>AGV3</t>
+  </si>
+  <si>
+    <t>AGV4</t>
+  </si>
+  <si>
+    <t>AGV5</t>
+  </si>
+  <si>
+    <t>AGV6</t>
+  </si>
+  <si>
+    <t>M1190</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M1191</t>
+  </si>
+  <si>
+    <t>M1192</t>
+  </si>
+  <si>
+    <t>M1193</t>
+  </si>
+  <si>
+    <t>M1194</t>
+  </si>
+  <si>
+    <t>M1195</t>
+  </si>
+  <si>
+    <t>M1196</t>
+  </si>
+  <si>
+    <t>M1197</t>
+  </si>
+  <si>
+    <t>M2228</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M2229</t>
+  </si>
+  <si>
+    <t>M2230</t>
+  </si>
+  <si>
+    <t>M2231</t>
+  </si>
+  <si>
+    <t>M2232</t>
+  </si>
+  <si>
+    <t>D01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV1 기동 MAIN 신호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV2 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>AGV3 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>AGV4 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>AGV5 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>AGV6 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>AGV7 기동 MAIN 신호</t>
+  </si>
+  <si>
+    <t>T40</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV1 기동 MAIN 딜레이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M150</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M151</t>
+  </si>
+  <si>
+    <t>M152</t>
+  </si>
+  <si>
+    <t>M153</t>
+  </si>
+  <si>
+    <t>M154</t>
+  </si>
+  <si>
+    <t>M155</t>
+  </si>
+  <si>
+    <t>M156</t>
+  </si>
+  <si>
+    <t>경유지점
+P[1~2]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1번 배터리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2번 배터리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3번 배터리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4번 배터리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1번 커버</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2번 커버</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>볼트 체결</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경유지점
+P[0]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1번 판</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2번 판</t>
   </si>
   <si>
     <t>하우징
 대차
+P[3~4]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1-&gt;3-&gt;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV
+P[5]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2-&gt;4-&gt;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1-&gt;3-&gt;4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>셀 대차
+P[3,5]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경유지점
 P[2]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>1-&gt;5-&gt;6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>AGV
-P[2]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2공정(접착제)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>6공정(접착제)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>8공정(접착제)</t>
+P[4,6]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2-&gt;7-&gt;4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>셀 대차
+P[7,8]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2-&gt;8-&gt;6</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>AGV
-P[2~5]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>볼트공급
-P[2]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M300</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M301</t>
-  </si>
-  <si>
-    <t>M302</t>
-  </si>
-  <si>
-    <t>M303</t>
-  </si>
-  <si>
-    <t>M304</t>
-  </si>
-  <si>
-    <t>M305</t>
-  </si>
-  <si>
-    <t>M306</t>
-  </si>
-  <si>
-    <t>M307</t>
-  </si>
-  <si>
-    <t>M308</t>
-  </si>
-  <si>
-    <t>M309</t>
-  </si>
-  <si>
-    <t>M310</t>
-  </si>
-  <si>
-    <t>M311</t>
-  </si>
-  <si>
-    <t>M312</t>
-  </si>
-  <si>
-    <t>M313</t>
-  </si>
-  <si>
-    <t>경화1 공정 완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정1 AGV 배출 신호</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정1 완료 후 문닫힘</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화2 공정 완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정2 AGV 배출 신호</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정2 완료 후 문닫힘</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화3 공정 완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정3 AGV 배출 신호</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>경화공정3 완료 후 문닫힘</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M120</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M121</t>
-  </si>
-  <si>
-    <t>M122</t>
-  </si>
-  <si>
-    <t>M123</t>
-  </si>
-  <si>
-    <t>M124</t>
-  </si>
-  <si>
-    <t>M125</t>
-  </si>
-  <si>
-    <t>M126</t>
-  </si>
-  <si>
-    <t>M127</t>
-  </si>
-  <si>
-    <t>M128</t>
-  </si>
-  <si>
-    <t>AGV 내부 펄스</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>T20</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>T21</t>
-  </si>
-  <si>
-    <t>T22</t>
-  </si>
-  <si>
-    <t>T23</t>
-  </si>
-  <si>
-    <t>T24</t>
-  </si>
-  <si>
-    <t>T25</t>
-  </si>
-  <si>
-    <t>T26</t>
-  </si>
-  <si>
-    <t>T27</t>
-  </si>
-  <si>
-    <t>T28</t>
-  </si>
-  <si>
-    <t>T29</t>
-  </si>
-  <si>
-    <t>1공정 agv 신호 딜레이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>3공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>4공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>5공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>6공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>7공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>8공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>9공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>10공정 agv 신호 딜레이</t>
-  </si>
-  <si>
-    <t>M129</t>
-  </si>
-  <si>
-    <t>프레스1(제4공정_저항 검사 공정)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>프레스2(제1공정_하우징 공정)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>로봇1 작업완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>로봇2 작업완료</t>
-  </si>
-  <si>
-    <t>로봇3 작업완료</t>
-  </si>
-  <si>
-    <t>로봇5 작업완료</t>
-  </si>
-  <si>
-    <t>로봇6 작업완료</t>
-  </si>
-  <si>
-    <t>로봇7 작업완료</t>
-  </si>
-  <si>
-    <t>로봇8 작업완료</t>
-  </si>
-  <si>
-    <t>로봇9 작업완료</t>
-  </si>
-  <si>
-    <t>프레스 작업완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>챔버1 상태</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M11</t>
-  </si>
-  <si>
-    <t>M12</t>
-  </si>
-  <si>
-    <t>M13</t>
-  </si>
-  <si>
-    <t>챔버2 상태</t>
-  </si>
-  <si>
-    <t>챔버3 상태</t>
-  </si>
-  <si>
-    <t>챔버4 상태</t>
-  </si>
-  <si>
-    <t>T30</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>챔버1 완료 후 딜레이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>T31</t>
-  </si>
-  <si>
-    <t>T32</t>
-  </si>
-  <si>
-    <t>T33</t>
-  </si>
-  <si>
-    <t>챔버2 완료 후 딜레이</t>
-  </si>
-  <si>
-    <t>챔버3 완료 후 딜레이</t>
-  </si>
-  <si>
-    <t>챔버4 완료 후 딜레이</t>
-  </si>
-  <si>
-    <t>M15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M16</t>
-  </si>
-  <si>
-    <t>M17</t>
-  </si>
-  <si>
-    <t>M18</t>
-  </si>
-  <si>
-    <t>챔버1 로봇 경유위치 이동 완료</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>챔버2 로봇 경유위치 이동 완료</t>
-  </si>
-  <si>
-    <t>챔버3 로봇 경유위치 이동 완료</t>
-  </si>
-  <si>
-    <t>챔버4 로봇 경유위치 이동 완료</t>
-  </si>
-  <si>
-    <t>M20</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>수작업7 START</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M21</t>
-  </si>
-  <si>
-    <t>M22</t>
-  </si>
-  <si>
-    <t>수작업8 START</t>
-  </si>
-  <si>
-    <t>수작업9 START</t>
-  </si>
-  <si>
-    <t>출하장</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PASS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NG</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M90</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGV1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M91</t>
-  </si>
-  <si>
-    <t>M92</t>
-  </si>
-  <si>
-    <t>M93</t>
-  </si>
-  <si>
-    <t>M94</t>
-  </si>
-  <si>
-    <t>M95</t>
-  </si>
-  <si>
-    <t>AGV2</t>
-  </si>
-  <si>
-    <t>AGV3</t>
-  </si>
-  <si>
-    <t>AGV4</t>
-  </si>
-  <si>
-    <t>AGV5</t>
-  </si>
-  <si>
-    <t>AGV6</t>
-  </si>
-  <si>
-    <t>M1190</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M1191</t>
-  </si>
-  <si>
-    <t>M1192</t>
-  </si>
-  <si>
-    <t>M1193</t>
-  </si>
-  <si>
-    <t>M1194</t>
-  </si>
-  <si>
-    <t>M1195</t>
-  </si>
-  <si>
-    <t>M1196</t>
-  </si>
-  <si>
-    <t>M1197</t>
-  </si>
-  <si>
-    <t>M2228</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M2229</t>
-  </si>
-  <si>
-    <t>M2230</t>
-  </si>
-  <si>
-    <t>M2231</t>
-  </si>
-  <si>
-    <t>M2232</t>
-  </si>
-  <si>
-    <t>D01</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGV1 기동 MAIN 신호</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGV2 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>AGV3 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>AGV4 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>AGV5 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>AGV6 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>AGV7 기동 MAIN 신호</t>
-  </si>
-  <si>
-    <t>T40</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGV1 기동 MAIN 딜레이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M150</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>M151</t>
-  </si>
-  <si>
-    <t>M152</t>
-  </si>
-  <si>
-    <t>M153</t>
-  </si>
-  <si>
-    <t>M154</t>
-  </si>
-  <si>
-    <t>M155</t>
-  </si>
-  <si>
-    <t>M156</t>
-  </si>
-  <si>
-    <t>경유지점
-P[1~2]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1번 배터리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2번 배터리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3번 배터리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4번 배터리</t>
+P[1~24]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV
+P[1~19]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1-&gt;2-&gt;3-&gt;1-&gt;4-&gt;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1-&gt;2-&gt;4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>셀 대차
+P[2~3]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGV
+P[4]
 P[3~6]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>1-&gt;2-&gt;3-&gt;2-&gt;4-&gt;2-&gt;5-&gt;2-&gt;6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>AGV
-P[7~8]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1-&gt;3-&gt;7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2-&gt;4-&gt;8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2-&gt;6-&gt;8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1-&gt;5-&gt;7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1번 커버</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2번 커버</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>셀 대차
-P[3~4]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1-&gt;3-.5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2-&gt;4-&gt;6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGV
-P[3~6]
-P[5~6]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>볼트 체결</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1-&gt;2-&gt;3~6</t>
+P[1~8]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3294,7 +3334,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -3701,13 +3741,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3807,17 +3873,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3915,6 +3972,12 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3928,12 +3991,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3951,8 +4008,29 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4302,47 +4380,47 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:11">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="33" t="s">
+      <c r="C3" s="80"/>
+      <c r="D3" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
     </row>
     <row r="4" spans="2:11">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="2:11">
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="80"/>
       <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="35"/>
+      <c r="F5" s="80"/>
       <c r="G5" s="4" t="s">
         <v>10</v>
       </c>
@@ -4513,7 +4591,7 @@
         <v>121</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>448</v>
@@ -4539,7 +4617,7 @@
         <v>122</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>450</v>
@@ -4565,7 +4643,7 @@
         <v>123</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>448</v>
@@ -4591,7 +4669,7 @@
         <v>124</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>450</v>
@@ -4631,10 +4709,10 @@
         <v>126</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="6"/>
@@ -4655,10 +4733,10 @@
         <v>127</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>798</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>801</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>509</v>
@@ -4683,10 +4761,10 @@
         <v>52</v>
       </c>
       <c r="H18" s="5" t="s">
+        <v>796</v>
+      </c>
+      <c r="I18" s="6" t="s">
         <v>799</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>802</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>510</v>
@@ -4713,10 +4791,10 @@
         <v>132</v>
       </c>
       <c r="H19" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="I19" s="6" t="s">
         <v>800</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>803</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>511</v>
@@ -4787,16 +4865,16 @@
         <v>135</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="I22" s="32" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
     </row>
     <row r="23" spans="2:11">
@@ -4817,16 +4895,16 @@
         <v>136</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
     </row>
     <row r="24" spans="2:11">
@@ -4847,16 +4925,16 @@
         <v>137</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="I24" s="32" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
     </row>
     <row r="25" spans="2:11">
@@ -4875,16 +4953,16 @@
         <v>170</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="I25" s="32" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
     </row>
     <row r="26" spans="2:11">
@@ -4905,10 +4983,10 @@
       <c r="H26" s="5"/>
       <c r="I26" s="6"/>
       <c r="J26" s="5" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
     </row>
     <row r="27" spans="2:11">
@@ -4929,10 +5007,10 @@
       <c r="H27" s="5"/>
       <c r="I27" s="6"/>
       <c r="J27" s="5" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
     </row>
     <row r="28" spans="2:11">
@@ -4953,16 +5031,16 @@
         <v>173</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
     </row>
     <row r="29" spans="2:11">
@@ -4983,16 +5061,16 @@
         <v>174</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
     </row>
     <row r="30" spans="2:11">
@@ -5013,16 +5091,16 @@
         <v>175</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
     </row>
     <row r="31" spans="2:11">
@@ -5045,10 +5123,10 @@
       <c r="H31" s="5"/>
       <c r="I31" s="6"/>
       <c r="J31" s="5" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
     </row>
     <row r="32" spans="2:11">
@@ -5093,10 +5171,10 @@
       <c r="H33" s="5"/>
       <c r="I33" s="6"/>
       <c r="J33" s="5" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="34" spans="2:11">
@@ -5117,10 +5195,10 @@
       <c r="H34" s="5"/>
       <c r="I34" s="6"/>
       <c r="J34" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="K34" s="6" t="s">
         <v>806</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="35" spans="2:11">
@@ -5145,10 +5223,10 @@
         <v>474</v>
       </c>
       <c r="J35" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="K35" s="6" t="s">
         <v>807</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="36" spans="2:11">
@@ -5173,10 +5251,10 @@
         <v>475</v>
       </c>
       <c r="J36" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="K36" s="6" t="s">
         <v>808</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="37" spans="2:11">
@@ -5249,10 +5327,10 @@
         <v>478</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
     </row>
     <row r="40" spans="2:11">
@@ -5411,10 +5489,10 @@
         <v>191</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="J46" s="5"/>
       <c r="K46" s="6"/>
@@ -5435,10 +5513,10 @@
         <v>192</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="J47" s="5"/>
       <c r="K47" s="6"/>
@@ -5459,10 +5537,10 @@
         <v>193</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="J48" s="5"/>
       <c r="K48" s="6"/>
@@ -5479,10 +5557,10 @@
         <v>194</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="J49" s="5"/>
       <c r="K49" s="6"/>
@@ -5499,10 +5577,10 @@
         <v>195</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="J50" s="5"/>
       <c r="K50" s="6"/>
@@ -5519,10 +5597,10 @@
         <v>196</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="J51" s="5"/>
       <c r="K51" s="6"/>
@@ -5559,10 +5637,10 @@
         <v>376</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="J53" s="5"/>
       <c r="K53" s="6"/>
@@ -5581,10 +5659,10 @@
         <v>377</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="J54" s="5"/>
       <c r="K54" s="6"/>
@@ -5603,10 +5681,10 @@
         <v>378</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="J55" s="5"/>
       <c r="K55" s="6"/>
@@ -5625,10 +5703,10 @@
         <v>379</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="J56" s="5"/>
       <c r="K56" s="6"/>
@@ -5647,10 +5725,10 @@
         <v>380</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="J57" s="5"/>
       <c r="K57" s="6"/>
@@ -5659,10 +5737,10 @@
       <c r="F58" s="5"/>
       <c r="G58" s="6"/>
       <c r="H58" s="5" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="6"/>
@@ -5671,10 +5749,10 @@
       <c r="F59" s="5"/>
       <c r="G59" s="6"/>
       <c r="H59" s="5" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
@@ -5859,84 +5937,84 @@
       <c r="F77" s="5"/>
       <c r="G77" s="6"/>
       <c r="H77" s="5" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="J77" s="6"/>
       <c r="K77" s="6"/>
     </row>
     <row r="78" spans="6:11">
       <c r="H78" s="5" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="79" spans="6:11">
       <c r="H79" s="5" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
     </row>
     <row r="80" spans="6:11">
       <c r="H80" s="5" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="81" spans="8:9">
       <c r="H81" s="5" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
     </row>
     <row r="82" spans="8:9">
       <c r="H82" s="5" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
     </row>
     <row r="83" spans="8:9">
       <c r="H83" s="5" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
     </row>
     <row r="84" spans="8:9">
       <c r="H84" s="5" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
     </row>
     <row r="85" spans="8:9">
       <c r="H85" s="5" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="I85" s="6" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
     </row>
     <row r="86" spans="8:9">
       <c r="H86" s="5" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="I86" s="6" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
     </row>
     <row r="87" spans="8:9">
@@ -5957,120 +6035,120 @@
     </row>
     <row r="91" spans="8:9">
       <c r="H91" s="5" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="I91" s="6" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="92" spans="8:9">
       <c r="H92" s="5" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="I92" s="6" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="93" spans="8:9">
       <c r="H93" s="5" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="I93" s="6" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
     </row>
     <row r="94" spans="8:9">
       <c r="H94" s="5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="I94" s="6" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
     </row>
     <row r="95" spans="8:9">
       <c r="H95" s="5" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="I95" s="6" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
     </row>
     <row r="96" spans="8:9">
       <c r="H96" s="5" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="I96" s="6" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
     </row>
     <row r="97" spans="8:9">
       <c r="H97" s="5" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="I97" s="6" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="98" spans="8:9">
       <c r="H98" s="5" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="I98" s="6" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
     </row>
     <row r="99" spans="8:9">
       <c r="H99" s="5" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="I99" s="6" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
     </row>
     <row r="100" spans="8:9">
       <c r="H100" s="5" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="I100" s="6" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="101" spans="8:9">
       <c r="H101" s="5" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="102" spans="8:9">
       <c r="H102" s="5" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="I102" s="6" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
     </row>
     <row r="103" spans="8:9">
       <c r="H103" s="5" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="I103" s="6" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="104" spans="8:9">
       <c r="H104" s="5" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="I104" s="6" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="105" spans="8:9">
       <c r="H105" s="5"/>
       <c r="I105" s="6" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
     </row>
   </sheetData>
@@ -6131,105 +6209,105 @@
       <c r="X2" s="12"/>
     </row>
     <row r="3" spans="3:24" s="3" customFormat="1">
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33" t="s">
+      <c r="D3" s="78"/>
+      <c r="E3" s="78" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="K3" s="33" t="s">
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="K3" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33" t="s">
+      <c r="L3" s="78"/>
+      <c r="M3" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="S3" s="33" t="s">
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
+      <c r="S3" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="33"/>
-      <c r="U3" s="33" t="s">
+      <c r="T3" s="78"/>
+      <c r="U3" s="78" t="s">
         <v>209</v>
       </c>
-      <c r="V3" s="33"/>
-      <c r="W3" s="33"/>
-      <c r="X3" s="33"/>
+      <c r="V3" s="78"/>
+      <c r="W3" s="78"/>
+      <c r="X3" s="78"/>
     </row>
     <row r="4" spans="3:24" s="3" customFormat="1">
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="33" t="s">
+      <c r="K4" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="S4" s="33" t="s">
+      <c r="L4" s="78"/>
+      <c r="M4" s="78"/>
+      <c r="N4" s="78"/>
+      <c r="O4" s="78"/>
+      <c r="P4" s="78"/>
+      <c r="S4" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="T4" s="33"/>
-      <c r="U4" s="33"/>
-      <c r="V4" s="33"/>
-      <c r="W4" s="33"/>
-      <c r="X4" s="33"/>
+      <c r="T4" s="78"/>
+      <c r="U4" s="78"/>
+      <c r="V4" s="78"/>
+      <c r="W4" s="78"/>
+      <c r="X4" s="78"/>
     </row>
     <row r="5" spans="3:24" s="2" customFormat="1">
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="33"/>
+      <c r="D5" s="78"/>
       <c r="E5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="33" t="s">
+      <c r="F5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="33"/>
+      <c r="G5" s="78"/>
       <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="33" t="s">
+      <c r="K5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="33"/>
+      <c r="L5" s="78"/>
       <c r="M5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N5" s="33" t="s">
+      <c r="N5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="O5" s="33"/>
+      <c r="O5" s="78"/>
       <c r="P5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="S5" s="33" t="s">
+      <c r="S5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="T5" s="33"/>
+      <c r="T5" s="78"/>
       <c r="U5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="V5" s="33" t="s">
+      <c r="V5" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="W5" s="33"/>
+      <c r="W5" s="78"/>
       <c r="X5" s="4" t="s">
         <v>10</v>
       </c>
@@ -6869,77 +6947,77 @@
       <c r="B23" s="1"/>
       <c r="E23" s="1"/>
       <c r="H23" s="1"/>
-      <c r="K23" s="33" t="s">
+      <c r="K23" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33" t="s">
+      <c r="L23" s="78"/>
+      <c r="M23" s="78" t="s">
         <v>210</v>
       </c>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
-      <c r="P23" s="33"/>
-      <c r="S23" s="33" t="s">
+      <c r="N23" s="78"/>
+      <c r="O23" s="78"/>
+      <c r="P23" s="78"/>
+      <c r="S23" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="T23" s="33"/>
-      <c r="U23" s="33" t="s">
+      <c r="T23" s="78"/>
+      <c r="U23" s="78" t="s">
         <v>211</v>
       </c>
-      <c r="V23" s="33"/>
-      <c r="W23" s="33"/>
-      <c r="X23" s="33"/>
+      <c r="V23" s="78"/>
+      <c r="W23" s="78"/>
+      <c r="X23" s="78"/>
     </row>
     <row r="24" spans="2:24">
       <c r="B24" s="1"/>
       <c r="E24" s="1"/>
       <c r="H24" s="1"/>
-      <c r="K24" s="33" t="s">
+      <c r="K24" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
-      <c r="S24" s="33" t="s">
+      <c r="L24" s="78"/>
+      <c r="M24" s="78"/>
+      <c r="N24" s="78"/>
+      <c r="O24" s="78"/>
+      <c r="P24" s="78"/>
+      <c r="S24" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="T24" s="33"/>
-      <c r="U24" s="33"/>
-      <c r="V24" s="33"/>
-      <c r="W24" s="33"/>
-      <c r="X24" s="33"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="78"/>
+      <c r="V24" s="78"/>
+      <c r="W24" s="78"/>
+      <c r="X24" s="78"/>
     </row>
     <row r="25" spans="2:24">
       <c r="B25" s="1"/>
       <c r="E25" s="1"/>
       <c r="H25" s="1"/>
-      <c r="K25" s="33" t="s">
+      <c r="K25" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="L25" s="33"/>
+      <c r="L25" s="78"/>
       <c r="M25" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N25" s="33" t="s">
+      <c r="N25" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="O25" s="33"/>
+      <c r="O25" s="78"/>
       <c r="P25" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="S25" s="33" t="s">
+      <c r="S25" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="T25" s="33"/>
+      <c r="T25" s="78"/>
       <c r="U25" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="V25" s="33" t="s">
+      <c r="V25" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="W25" s="33"/>
+      <c r="W25" s="78"/>
       <c r="X25" s="4" t="s">
         <v>10</v>
       </c>
@@ -7399,114 +7477,114 @@
     </row>
     <row r="42" spans="2:24">
       <c r="B42" s="8"/>
-      <c r="C42" s="33" t="s">
+      <c r="C42" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33" t="s">
+      <c r="D42" s="78"/>
+      <c r="E42" s="78" t="s">
         <v>212</v>
       </c>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
+      <c r="F42" s="78"/>
+      <c r="G42" s="78"/>
+      <c r="H42" s="78"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
       <c r="K42" s="4" t="s">
         <v>40</v>
       </c>
       <c r="L42" s="4"/>
-      <c r="M42" s="33" t="s">
+      <c r="M42" s="78" t="s">
         <v>213</v>
       </c>
-      <c r="N42" s="33"/>
-      <c r="O42" s="33"/>
-      <c r="P42" s="33"/>
+      <c r="N42" s="78"/>
+      <c r="O42" s="78"/>
+      <c r="P42" s="78"/>
       <c r="Q42" s="8"/>
       <c r="S42" s="4" t="s">
         <v>40</v>
       </c>
       <c r="T42" s="4"/>
-      <c r="U42" s="33" t="s">
+      <c r="U42" s="78" t="s">
         <v>214</v>
       </c>
-      <c r="V42" s="33"/>
-      <c r="W42" s="33"/>
-      <c r="X42" s="33"/>
+      <c r="V42" s="78"/>
+      <c r="W42" s="78"/>
+      <c r="X42" s="78"/>
     </row>
     <row r="43" spans="2:24">
       <c r="B43" s="8"/>
-      <c r="C43" s="33" t="s">
+      <c r="C43" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="D43" s="33"/>
-      <c r="E43" s="33"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="33"/>
-      <c r="H43" s="33"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="78"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="78"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
       <c r="K43" s="4" t="s">
         <v>39</v>
       </c>
       <c r="L43" s="4"/>
-      <c r="M43" s="33"/>
-      <c r="N43" s="33"/>
-      <c r="O43" s="33"/>
-      <c r="P43" s="33"/>
+      <c r="M43" s="78"/>
+      <c r="N43" s="78"/>
+      <c r="O43" s="78"/>
+      <c r="P43" s="78"/>
       <c r="Q43" s="8"/>
       <c r="S43" s="4" t="s">
         <v>39</v>
       </c>
       <c r="T43" s="4"/>
-      <c r="U43" s="33"/>
-      <c r="V43" s="33"/>
-      <c r="W43" s="33"/>
-      <c r="X43" s="33"/>
+      <c r="U43" s="78"/>
+      <c r="V43" s="78"/>
+      <c r="W43" s="78"/>
+      <c r="X43" s="78"/>
     </row>
     <row r="44" spans="2:24">
       <c r="B44" s="8"/>
-      <c r="C44" s="33" t="s">
+      <c r="C44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="D44" s="33"/>
+      <c r="D44" s="78"/>
       <c r="E44" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F44" s="33" t="s">
+      <c r="F44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="G44" s="33"/>
+      <c r="G44" s="78"/>
       <c r="H44" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
-      <c r="K44" s="33" t="s">
+      <c r="K44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="L44" s="33"/>
+      <c r="L44" s="78"/>
       <c r="M44" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N44" s="33" t="s">
+      <c r="N44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="O44" s="33"/>
+      <c r="O44" s="78"/>
       <c r="P44" s="4" t="s">
         <v>10</v>
       </c>
       <c r="Q44" s="8"/>
-      <c r="S44" s="33" t="s">
+      <c r="S44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="T44" s="33"/>
+      <c r="T44" s="78"/>
       <c r="U44" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="V44" s="33" t="s">
+      <c r="V44" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="W44" s="33"/>
+      <c r="W44" s="78"/>
       <c r="X44" s="4" t="s">
         <v>10</v>
       </c>
@@ -7939,7 +8017,7 @@
         <v>620</v>
       </c>
       <c r="U52" s="10" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="V52" s="9" t="s">
         <v>327</v>
@@ -7999,7 +8077,7 @@
         <v>621</v>
       </c>
       <c r="U53" s="10" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="V53" s="9" t="s">
         <v>259</v>
@@ -8224,29 +8302,29 @@
       </c>
     </row>
     <row r="3" spans="2:21">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="34" t="s">
-        <v>782</v>
-      </c>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="35"/>
-      <c r="I3" s="34" t="s">
+      <c r="C3" s="80"/>
+      <c r="D3" s="79" t="s">
+        <v>779</v>
+      </c>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="80"/>
+      <c r="I3" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="J3" s="35"/>
-      <c r="K3" s="33" t="s">
+      <c r="J3" s="80"/>
+      <c r="K3" s="78" t="s">
         <v>302</v>
       </c>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="33"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="78"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
+      <c r="Q3" s="78"/>
       <c r="S3" s="5">
         <v>0</v>
       </c>
@@ -8256,25 +8334,25 @@
       <c r="U3" s="6"/>
     </row>
     <row r="4" spans="2:21">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="35"/>
-      <c r="I4" s="34" t="s">
+      <c r="C4" s="80"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="80"/>
+      <c r="I4" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="35"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="33"/>
+      <c r="J4" s="80"/>
+      <c r="K4" s="78"/>
+      <c r="L4" s="78"/>
+      <c r="M4" s="78"/>
+      <c r="N4" s="78"/>
+      <c r="O4" s="78"/>
+      <c r="P4" s="78"/>
+      <c r="Q4" s="78"/>
       <c r="S4" s="5">
         <v>100</v>
       </c>
@@ -8286,38 +8364,38 @@
       </c>
     </row>
     <row r="5" spans="2:21">
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="35"/>
+      <c r="C5" s="80"/>
       <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="35"/>
+      <c r="F5" s="80"/>
       <c r="G5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="34" t="s">
+      <c r="I5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="35"/>
+      <c r="J5" s="80"/>
       <c r="K5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="34" t="s">
+      <c r="L5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="M5" s="35"/>
+      <c r="M5" s="80"/>
       <c r="N5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="34" t="s">
+      <c r="O5" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="P5" s="35"/>
+      <c r="P5" s="80"/>
       <c r="Q5" s="4" t="s">
         <v>10</v>
       </c>
@@ -8850,16 +8928,16 @@
       </c>
     </row>
     <row r="20" spans="2:21">
-      <c r="B20" s="33" t="s">
+      <c r="B20" s="78" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33" t="s">
-        <v>781</v>
-      </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="78" t="s">
+        <v>778</v>
+      </c>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
       <c r="K20" s="6"/>
@@ -8880,14 +8958,14 @@
       </c>
     </row>
     <row r="21" spans="2:21">
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="6"/>
@@ -8908,17 +8986,17 @@
       </c>
     </row>
     <row r="22" spans="2:21">
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="33"/>
+      <c r="C22" s="78"/>
       <c r="D22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="33" t="s">
+      <c r="E22" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="33"/>
+      <c r="F22" s="78"/>
       <c r="G22" s="4" t="s">
         <v>10</v>
       </c>
@@ -9112,19 +9190,19 @@
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
       <c r="G28" s="10"/>
-      <c r="I28" s="34" t="s">
+      <c r="I28" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="J28" s="35"/>
-      <c r="K28" s="33" t="s">
+      <c r="J28" s="80"/>
+      <c r="K28" s="78" t="s">
         <v>302</v>
       </c>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="33"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
+      <c r="L28" s="78"/>
+      <c r="M28" s="78"/>
+      <c r="N28" s="78"/>
+      <c r="O28" s="78"/>
+      <c r="P28" s="78"/>
+      <c r="Q28" s="78"/>
       <c r="S28" s="5">
         <v>1400</v>
       </c>
@@ -9146,22 +9224,22 @@
         <v>645</v>
       </c>
       <c r="G29" s="10"/>
-      <c r="I29" s="34" t="s">
+      <c r="I29" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="J29" s="35"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
-      <c r="N29" s="33"/>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33"/>
-      <c r="Q29" s="33"/>
+      <c r="J29" s="80"/>
+      <c r="K29" s="78"/>
+      <c r="L29" s="78"/>
+      <c r="M29" s="78"/>
+      <c r="N29" s="78"/>
+      <c r="O29" s="78"/>
+      <c r="P29" s="78"/>
+      <c r="Q29" s="78"/>
       <c r="S29" s="5">
         <v>1500</v>
       </c>
       <c r="T29" s="6" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="U29" s="6"/>
     </row>
@@ -9178,24 +9256,24 @@
       <c r="G30" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I30" s="34" t="s">
+      <c r="I30" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="J30" s="35"/>
+      <c r="J30" s="80"/>
       <c r="K30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L30" s="34" t="s">
+      <c r="L30" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="M30" s="35"/>
+      <c r="M30" s="80"/>
       <c r="N30" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O30" s="34" t="s">
+      <c r="O30" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="P30" s="35"/>
+      <c r="P30" s="80"/>
       <c r="Q30" s="4" t="s">
         <v>10</v>
       </c>
@@ -9244,20 +9322,20 @@
       <c r="G32" s="10"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>7</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="5" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="N32" s="6" t="s">
         <v>20</v>
       </c>
       <c r="O32" s="16" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="P32" s="16"/>
       <c r="Q32" s="6" t="s">
@@ -9279,14 +9357,14 @@
       <c r="G33" s="10"/>
       <c r="I33" s="9"/>
       <c r="J33" s="9" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="K33" s="10" t="s">
         <v>317</v>
       </c>
       <c r="L33" s="9"/>
       <c r="M33" s="9" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="N33" s="10" t="s">
         <v>13</v>
@@ -9304,14 +9382,14 @@
       <c r="G34" s="12"/>
       <c r="I34" s="9"/>
       <c r="J34" s="9" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="K34" s="10" t="s">
         <v>318</v>
       </c>
       <c r="L34" s="9"/>
       <c r="M34" s="9" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="N34" s="10" t="s">
         <v>14</v>
@@ -9323,14 +9401,14 @@
     <row r="35" spans="2:17">
       <c r="I35" s="9"/>
       <c r="J35" s="9" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="K35" s="10" t="s">
         <v>17</v>
       </c>
       <c r="L35" s="9"/>
       <c r="M35" s="9" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="N35" s="10" t="s">
         <v>316</v>
@@ -9342,14 +9420,14 @@
     <row r="36" spans="2:17">
       <c r="I36" s="9"/>
       <c r="J36" s="9" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="K36" s="10" t="s">
         <v>18</v>
       </c>
       <c r="L36" s="9"/>
       <c r="M36" s="9" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="N36" s="10" t="s">
         <v>15</v>
@@ -9361,7 +9439,7 @@
     <row r="37" spans="2:17">
       <c r="I37" s="5"/>
       <c r="J37" s="5" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="K37" s="6"/>
       <c r="L37" s="5"/>
@@ -9374,7 +9452,7 @@
     <row r="38" spans="2:17">
       <c r="I38" s="5"/>
       <c r="J38" s="5" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>19</v>
@@ -9389,7 +9467,7 @@
     <row r="39" spans="2:17">
       <c r="I39" s="5"/>
       <c r="J39" s="5" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="K39" s="6" t="s">
         <v>385</v>
@@ -9550,64 +9628,77 @@
   <dimension ref="D3:X47"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
+    <col min="14" max="14" width="9.75" customWidth="1"/>
     <col min="15" max="15" width="12.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="4:20">
+      <c r="E3" t="s">
+        <v>877</v>
+      </c>
+      <c r="F3" t="s">
+        <v>880</v>
+      </c>
       <c r="N3" t="s">
+        <v>869</v>
+      </c>
+      <c r="O3" s="33" t="s">
+        <v>883</v>
+      </c>
+      <c r="P3" t="s">
+        <v>871</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="4" spans="4:20">
+      <c r="E4" t="s">
+        <v>878</v>
+      </c>
+      <c r="F4" t="s">
+        <v>882</v>
+      </c>
+      <c r="N4" t="s">
+        <v>870</v>
+      </c>
+      <c r="O4" s="33" t="s">
+        <v>886</v>
+      </c>
+      <c r="P4" t="s">
         <v>872</v>
       </c>
-      <c r="O3" s="81" t="s">
-        <v>878</v>
-      </c>
-      <c r="P3" t="s">
-        <v>874</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>881</v>
-      </c>
-    </row>
-    <row r="4" spans="4:20">
-      <c r="N4" t="s">
-        <v>873</v>
-      </c>
-      <c r="O4" s="81" t="s">
+      <c r="Q4" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="6" spans="4:20" ht="17.25" thickBot="1">
+      <c r="D6" s="68" t="s">
+        <v>357</v>
+      </c>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="I6" s="68" t="s">
+        <v>718</v>
+      </c>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="M6" s="68" t="s">
+        <v>359</v>
+      </c>
+      <c r="N6" s="68"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="68"/>
+      <c r="R6" s="68" t="s">
+        <v>719</v>
+      </c>
+      <c r="S6" s="68"/>
+      <c r="T6" s="68"/>
+    </row>
+    <row r="7" spans="4:20" ht="16.5" customHeight="1">
+      <c r="D7" s="34" t="s">
         <v>879</v>
-      </c>
-      <c r="P4" t="s">
-        <v>875</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>880</v>
-      </c>
-    </row>
-    <row r="6" spans="4:20" ht="17.25" thickBot="1">
-      <c r="D6" s="69" t="s">
-        <v>357</v>
-      </c>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="I6" s="69" t="s">
-        <v>721</v>
-      </c>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="M6" s="69" t="s">
-        <v>359</v>
-      </c>
-      <c r="N6" s="69"/>
-      <c r="O6" s="69"/>
-      <c r="P6" s="69"/>
-      <c r="R6" s="69" t="s">
-        <v>722</v>
-      </c>
-      <c r="S6" s="69"/>
-      <c r="T6" s="69"/>
-    </row>
-    <row r="7" spans="4:20" ht="16.5" customHeight="1">
-      <c r="D7" s="37" t="s">
-        <v>719</v>
       </c>
       <c r="E7" s="21"/>
       <c r="F7" s="21"/>
@@ -9615,206 +9706,212 @@
       <c r="I7" s="26"/>
       <c r="J7" s="21"/>
       <c r="K7" s="22"/>
-      <c r="M7" s="37" t="s">
-        <v>876</v>
+      <c r="M7" s="34" t="s">
+        <v>889</v>
       </c>
       <c r="N7" s="21"/>
       <c r="O7" s="21"/>
-      <c r="P7" s="22"/>
+      <c r="P7" s="34" t="s">
+        <v>884</v>
+      </c>
       <c r="R7" s="26"/>
       <c r="S7" s="21"/>
       <c r="T7" s="22"/>
     </row>
     <row r="8" spans="4:20">
-      <c r="D8" s="38"/>
+      <c r="D8" s="35"/>
       <c r="G8" s="23"/>
       <c r="I8" s="24"/>
       <c r="K8" s="23"/>
-      <c r="M8" s="38"/>
-      <c r="P8" s="23"/>
+      <c r="M8" s="35"/>
+      <c r="P8" s="35"/>
       <c r="R8" s="24"/>
       <c r="T8" s="23"/>
     </row>
     <row r="9" spans="4:20" ht="16.5" customHeight="1">
-      <c r="D9" s="38"/>
-      <c r="F9" s="49" t="s">
+      <c r="D9" s="35"/>
+      <c r="F9" s="46" t="s">
         <v>717</v>
       </c>
       <c r="G9" s="23"/>
       <c r="I9" s="24"/>
-      <c r="J9" s="49" t="s">
+      <c r="J9" s="46" t="s">
         <v>717</v>
       </c>
       <c r="K9" s="23"/>
-      <c r="M9" s="38"/>
-      <c r="O9" s="49" t="s">
+      <c r="M9" s="35"/>
+      <c r="O9" s="84" t="s">
         <v>717</v>
       </c>
-      <c r="P9" s="23"/>
+      <c r="P9" s="35"/>
       <c r="R9" s="24"/>
-      <c r="S9" s="49" t="s">
+      <c r="S9" s="46" t="s">
         <v>717</v>
       </c>
       <c r="T9" s="23"/>
     </row>
     <row r="10" spans="4:20">
-      <c r="D10" s="38"/>
-      <c r="F10" s="50"/>
+      <c r="D10" s="35"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="23"/>
       <c r="I10" s="24"/>
-      <c r="J10" s="50"/>
+      <c r="J10" s="47"/>
       <c r="K10" s="23"/>
-      <c r="M10" s="38"/>
-      <c r="O10" s="50"/>
-      <c r="P10" s="23"/>
+      <c r="M10" s="35"/>
+      <c r="O10" s="85"/>
+      <c r="P10" s="35"/>
       <c r="R10" s="24"/>
-      <c r="S10" s="50"/>
+      <c r="S10" s="47"/>
       <c r="T10" s="23"/>
     </row>
-    <row r="11" spans="4:20" ht="16.5" customHeight="1">
-      <c r="D11" s="38"/>
-      <c r="E11" s="51" t="s">
-        <v>716</v>
+    <row r="11" spans="4:20">
+      <c r="D11" s="35"/>
+      <c r="E11" s="48" t="s">
+        <v>868</v>
       </c>
       <c r="G11" s="23"/>
       <c r="I11" s="24"/>
-      <c r="J11" s="51" t="s">
+      <c r="J11" s="48" t="s">
+        <v>876</v>
+      </c>
+      <c r="K11" s="23"/>
+      <c r="M11" s="35"/>
+      <c r="N11" s="48" t="s">
+        <v>885</v>
+      </c>
+      <c r="O11" s="82" t="s">
         <v>716</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="M11" s="38"/>
-      <c r="N11" s="51" t="s">
-        <v>871</v>
-      </c>
-      <c r="P11" s="23"/>
+      <c r="P11" s="35"/>
       <c r="R11" s="24"/>
-      <c r="S11" s="51" t="s">
-        <v>716</v>
+      <c r="S11" s="48" t="s">
+        <v>876</v>
       </c>
       <c r="T11" s="23"/>
     </row>
     <row r="12" spans="4:20">
-      <c r="D12" s="38"/>
-      <c r="E12" s="52"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="49"/>
       <c r="G12" s="23"/>
       <c r="I12" s="24"/>
-      <c r="J12" s="62"/>
+      <c r="J12" s="59"/>
       <c r="K12" s="23"/>
-      <c r="M12" s="38"/>
-      <c r="N12" s="52"/>
-      <c r="P12" s="23"/>
+      <c r="M12" s="35"/>
+      <c r="N12" s="49"/>
+      <c r="O12" s="83"/>
+      <c r="P12" s="35"/>
       <c r="R12" s="24"/>
-      <c r="S12" s="62"/>
+      <c r="S12" s="59"/>
       <c r="T12" s="23"/>
     </row>
     <row r="13" spans="4:20">
-      <c r="D13" s="39"/>
+      <c r="D13" s="36"/>
       <c r="G13" s="23"/>
       <c r="I13" s="24"/>
       <c r="K13" s="23"/>
-      <c r="M13" s="39"/>
-      <c r="P13" s="23"/>
+      <c r="M13" s="36"/>
+      <c r="P13" s="36"/>
       <c r="R13" s="24"/>
       <c r="T13" s="23"/>
     </row>
     <row r="14" spans="4:20" ht="16.5" customHeight="1">
       <c r="D14" s="24"/>
-      <c r="E14" s="40" t="s">
-        <v>718</v>
-      </c>
-      <c r="F14" s="41"/>
-      <c r="G14" s="42"/>
-      <c r="I14" s="53" t="s">
-        <v>724</v>
-      </c>
-      <c r="J14" s="54"/>
-      <c r="K14" s="55"/>
+      <c r="E14" s="37" t="s">
+        <v>881</v>
+      </c>
+      <c r="F14" s="38"/>
+      <c r="G14" s="39"/>
+      <c r="I14" s="50" t="s">
+        <v>892</v>
+      </c>
+      <c r="J14" s="51"/>
+      <c r="K14" s="52"/>
       <c r="M14" s="24"/>
-      <c r="N14" s="40" t="s">
-        <v>877</v>
-      </c>
-      <c r="O14" s="41"/>
-      <c r="P14" s="42"/>
-      <c r="R14" s="53" t="s">
-        <v>724</v>
-      </c>
-      <c r="S14" s="54"/>
-      <c r="T14" s="55"/>
+      <c r="N14" s="37" t="s">
+        <v>887</v>
+      </c>
+      <c r="O14" s="38"/>
+      <c r="P14" s="39"/>
+      <c r="R14" s="50" t="s">
+        <v>891</v>
+      </c>
+      <c r="S14" s="51"/>
+      <c r="T14" s="52"/>
     </row>
     <row r="15" spans="4:20">
       <c r="D15" s="24"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="45"/>
-      <c r="I15" s="56"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="58"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="42"/>
+      <c r="I15" s="53"/>
+      <c r="J15" s="54"/>
+      <c r="K15" s="55"/>
       <c r="M15" s="24"/>
-      <c r="N15" s="43"/>
-      <c r="O15" s="44"/>
-      <c r="P15" s="45"/>
-      <c r="R15" s="56"/>
-      <c r="S15" s="57"/>
-      <c r="T15" s="58"/>
+      <c r="N15" s="40"/>
+      <c r="O15" s="41"/>
+      <c r="P15" s="42"/>
+      <c r="R15" s="53"/>
+      <c r="S15" s="54"/>
+      <c r="T15" s="55"/>
     </row>
     <row r="16" spans="4:20">
       <c r="D16" s="24"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="45"/>
-      <c r="I16" s="56"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="58"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="42"/>
+      <c r="I16" s="53"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="55"/>
       <c r="M16" s="24"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="44"/>
-      <c r="P16" s="45"/>
-      <c r="R16" s="56"/>
-      <c r="S16" s="57"/>
-      <c r="T16" s="58"/>
+      <c r="N16" s="40"/>
+      <c r="O16" s="41"/>
+      <c r="P16" s="42"/>
+      <c r="R16" s="53"/>
+      <c r="S16" s="54"/>
+      <c r="T16" s="55"/>
     </row>
     <row r="17" spans="4:20" ht="17.25" thickBot="1">
       <c r="D17" s="25"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="47"/>
-      <c r="G17" s="48"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="61"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="45"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="58"/>
       <c r="M17" s="25"/>
-      <c r="N17" s="46"/>
-      <c r="O17" s="47"/>
-      <c r="P17" s="48"/>
-      <c r="R17" s="59"/>
-      <c r="S17" s="60"/>
-      <c r="T17" s="61"/>
+      <c r="N17" s="43"/>
+      <c r="O17" s="44"/>
+      <c r="P17" s="45"/>
+      <c r="R17" s="56"/>
+      <c r="S17" s="57"/>
+      <c r="T17" s="58"/>
     </row>
     <row r="19" spans="4:20" ht="17.25" thickBot="1">
-      <c r="D19" s="69" t="s">
+      <c r="D19" s="68" t="s">
         <v>368</v>
       </c>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="H19" s="69" t="s">
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="H19" s="68" t="s">
         <v>367</v>
       </c>
-      <c r="I19" s="69"/>
-      <c r="J19" s="69"/>
-      <c r="K19" s="69"/>
-      <c r="R19" s="69" t="s">
-        <v>723</v>
-      </c>
-      <c r="S19" s="69"/>
-      <c r="T19" s="69"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="68"/>
+      <c r="K19" s="68"/>
+      <c r="R19" s="68" t="s">
+        <v>720</v>
+      </c>
+      <c r="S19" s="68"/>
+      <c r="T19" s="68"/>
     </row>
     <row r="20" spans="4:20">
-      <c r="D20" s="77" t="s">
-        <v>720</v>
-      </c>
-      <c r="E20" s="78"/>
-      <c r="F20" s="79"/>
+      <c r="D20" s="74" t="s">
+        <v>898</v>
+      </c>
+      <c r="E20" s="75"/>
+      <c r="F20" s="76"/>
       <c r="H20" s="26"/>
-      <c r="I20" s="68" t="s">
+      <c r="I20" s="65" t="s">
         <v>717</v>
       </c>
       <c r="J20" s="21"/>
@@ -9823,56 +9920,56 @@
       <c r="N20" s="21"/>
       <c r="O20" s="21"/>
       <c r="P20" s="22"/>
-      <c r="R20" s="77" t="s">
-        <v>724</v>
-      </c>
-      <c r="S20" s="78"/>
-      <c r="T20" s="79"/>
+      <c r="R20" s="74" t="s">
+        <v>721</v>
+      </c>
+      <c r="S20" s="75"/>
+      <c r="T20" s="76"/>
     </row>
     <row r="21" spans="4:20">
-      <c r="D21" s="56"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="58"/>
+      <c r="D21" s="53"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="55"/>
       <c r="H21" s="24"/>
-      <c r="I21" s="50"/>
+      <c r="I21" s="47"/>
       <c r="K21" s="23"/>
       <c r="M21" s="24"/>
       <c r="P21" s="23"/>
-      <c r="R21" s="56"/>
-      <c r="S21" s="57"/>
-      <c r="T21" s="58"/>
+      <c r="R21" s="53"/>
+      <c r="S21" s="54"/>
+      <c r="T21" s="55"/>
     </row>
     <row r="22" spans="4:20">
-      <c r="D22" s="56"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="58"/>
-      <c r="H22" s="74" t="s">
-        <v>725</v>
-      </c>
-      <c r="I22" s="51" t="s">
+      <c r="D22" s="53"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="55"/>
+      <c r="H22" s="66" t="s">
+        <v>722</v>
+      </c>
+      <c r="I22" s="48" t="s">
         <v>716</v>
       </c>
-      <c r="J22" s="74"/>
+      <c r="J22" s="66"/>
       <c r="K22" s="23"/>
       <c r="M22" s="24"/>
       <c r="P22" s="23"/>
-      <c r="R22" s="56"/>
-      <c r="S22" s="57"/>
-      <c r="T22" s="58"/>
+      <c r="R22" s="53"/>
+      <c r="S22" s="54"/>
+      <c r="T22" s="55"/>
     </row>
     <row r="23" spans="4:20">
-      <c r="D23" s="65"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="80"/>
-      <c r="H23" s="75"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="75"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="77"/>
+      <c r="H23" s="67"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="67"/>
       <c r="K23" s="23"/>
       <c r="M23" s="24"/>
       <c r="P23" s="23"/>
-      <c r="R23" s="65"/>
-      <c r="S23" s="66"/>
-      <c r="T23" s="80"/>
+      <c r="R23" s="62"/>
+      <c r="S23" s="63"/>
+      <c r="T23" s="77"/>
     </row>
     <row r="24" spans="4:20">
       <c r="D24" s="24"/>
@@ -9888,77 +9985,77 @@
     </row>
     <row r="25" spans="4:20" ht="16.5" customHeight="1">
       <c r="D25" s="24"/>
-      <c r="E25" s="51" t="s">
-        <v>716</v>
+      <c r="E25" s="48" t="s">
+        <v>876</v>
       </c>
       <c r="F25" s="23"/>
-      <c r="H25" s="53" t="s">
-        <v>887</v>
-      </c>
-      <c r="I25" s="54"/>
-      <c r="J25" s="63"/>
+      <c r="H25" s="50" t="s">
+        <v>896</v>
+      </c>
+      <c r="I25" s="51"/>
+      <c r="J25" s="60"/>
       <c r="K25" s="23"/>
       <c r="M25" s="24"/>
       <c r="P25" s="23"/>
       <c r="R25" s="24"/>
-      <c r="S25" s="51" t="s">
+      <c r="S25" s="48" t="s">
         <v>716</v>
       </c>
       <c r="T25" s="23"/>
     </row>
     <row r="26" spans="4:20">
       <c r="D26" s="24"/>
-      <c r="E26" s="62"/>
+      <c r="E26" s="59"/>
       <c r="F26" s="23"/>
-      <c r="H26" s="56"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="64"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="54"/>
+      <c r="J26" s="61"/>
       <c r="K26" s="23"/>
       <c r="M26" s="24"/>
       <c r="P26" s="23"/>
       <c r="R26" s="24"/>
-      <c r="S26" s="62"/>
+      <c r="S26" s="59"/>
       <c r="T26" s="23"/>
     </row>
     <row r="27" spans="4:20">
       <c r="D27" s="24"/>
-      <c r="E27" s="49" t="s">
+      <c r="E27" s="46" t="s">
         <v>717</v>
       </c>
       <c r="F27" s="23"/>
-      <c r="H27" s="56"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="64"/>
-      <c r="K27" s="70" t="s">
-        <v>884</v>
+      <c r="H27" s="53"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="61"/>
+      <c r="K27" s="69" t="s">
+        <v>895</v>
       </c>
       <c r="M27" s="24"/>
       <c r="P27" s="23"/>
       <c r="R27" s="24"/>
-      <c r="S27" s="49" t="s">
+      <c r="S27" s="46" t="s">
         <v>717</v>
       </c>
       <c r="T27" s="23"/>
     </row>
     <row r="28" spans="4:20" ht="16.5" customHeight="1">
       <c r="D28" s="24"/>
-      <c r="E28" s="50"/>
+      <c r="E28" s="47"/>
       <c r="F28" s="23"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="67"/>
-      <c r="K28" s="71"/>
+      <c r="H28" s="62"/>
+      <c r="I28" s="63"/>
+      <c r="J28" s="64"/>
+      <c r="K28" s="70"/>
       <c r="M28" s="24"/>
       <c r="P28" s="23"/>
       <c r="R28" s="24"/>
-      <c r="S28" s="50"/>
+      <c r="S28" s="47"/>
       <c r="T28" s="23"/>
     </row>
     <row r="29" spans="4:20">
       <c r="D29" s="24"/>
       <c r="F29" s="23"/>
       <c r="H29" s="24"/>
-      <c r="K29" s="72"/>
+      <c r="K29" s="71"/>
       <c r="M29" s="24"/>
       <c r="P29" s="23"/>
       <c r="R29" s="24"/>
@@ -9969,10 +10066,10 @@
       <c r="E30" s="27"/>
       <c r="F30" s="28"/>
       <c r="H30" s="24"/>
-      <c r="I30" s="51" t="s">
-        <v>871</v>
-      </c>
-      <c r="K30" s="72"/>
+      <c r="I30" s="48" t="s">
+        <v>716</v>
+      </c>
+      <c r="K30" s="71"/>
       <c r="M30" s="25"/>
       <c r="N30" s="27"/>
       <c r="O30" s="27"/>
@@ -9983,53 +10080,56 @@
     </row>
     <row r="31" spans="4:20">
       <c r="H31" s="24"/>
-      <c r="I31" s="62"/>
-      <c r="K31" s="72"/>
+      <c r="I31" s="59"/>
+      <c r="K31" s="71"/>
     </row>
     <row r="32" spans="4:20">
       <c r="H32" s="24"/>
-      <c r="I32" s="49" t="s">
+      <c r="I32" s="46" t="s">
         <v>717</v>
       </c>
-      <c r="K32" s="72"/>
+      <c r="K32" s="71"/>
+      <c r="R32" t="s">
+        <v>893</v>
+      </c>
     </row>
     <row r="33" spans="8:24" ht="17.25" thickBot="1">
       <c r="H33" s="25"/>
-      <c r="I33" s="76"/>
+      <c r="I33" s="73"/>
       <c r="J33" s="27"/>
-      <c r="K33" s="73"/>
+      <c r="K33" s="72"/>
     </row>
     <row r="35" spans="8:24">
       <c r="I35" t="s">
-        <v>882</v>
+        <v>873</v>
       </c>
       <c r="J35" t="s">
-        <v>885</v>
+        <v>894</v>
       </c>
     </row>
     <row r="36" spans="8:24">
       <c r="I36" t="s">
+        <v>874</v>
+      </c>
+      <c r="J36" t="s">
         <v>883</v>
-      </c>
-      <c r="J36" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="38" spans="8:24">
       <c r="I38" t="s">
-        <v>888</v>
+        <v>875</v>
       </c>
       <c r="J38" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
     </row>
     <row r="47" spans="8:24">
       <c r="X47" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="37">
     <mergeCell ref="R6:T6"/>
     <mergeCell ref="R19:T19"/>
     <mergeCell ref="D19:F19"/>
@@ -10059,6 +10159,8 @@
     <mergeCell ref="O9:O10"/>
     <mergeCell ref="N11:N12"/>
     <mergeCell ref="N14:P17"/>
+    <mergeCell ref="P7:P13"/>
+    <mergeCell ref="O11:O12"/>
     <mergeCell ref="D7:D13"/>
     <mergeCell ref="E14:G17"/>
     <mergeCell ref="F9:F10"/>

</xml_diff>